<commit_message>
Fix Vercel build by removing scipy dependency
</commit_message>
<xml_diff>
--- a/FX_Hedging_Calculations.xlsx
+++ b/FX_Hedging_Calculations.xlsx
@@ -1700,16 +1700,16 @@
         <v>12476088.27632621</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>12485363.80924231</v>
+        <v>12485363.80924235</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>9275.532916106284</v>
+        <v>9275.532916147262</v>
       </c>
       <c r="J3" s="3" t="n">
-        <v>0.0007429125060208542</v>
+        <v>0.0007429125060241338</v>
       </c>
       <c r="K3" t="n">
-        <v>0.9260822460977648</v>
+        <v>0.9260822460977649</v>
       </c>
       <c r="L3" t="n">
         <v>0.04795811162363501</v>
@@ -1798,16 +1798,16 @@
         <v>15950594.42481099</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>15974569.14787114</v>
+        <v>15974569.14787112</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>23974.72306015342</v>
+        <v>23974.72306013107</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>0.001500805614112505</v>
+        <v>0.001500805614111108</v>
       </c>
       <c r="K5" t="n">
-        <v>0.7304175174656488</v>
+        <v>0.7304175174656486</v>
       </c>
       <c r="L5" t="n">
         <v>0.002721591769178966</v>

</xml_diff>